<commit_message>
Add ML validation script and outputs
Add new ML pipeline script UTR221_ML_validacao3.py that loads urt220/urt221 data, performs feature engineering, trains a RandomForest regressor, and runs evaluations. Implements recursive validation and failure simulation, and generates DF1-DF6 Excel exports (DF2_sem_zeros.xlsx, DF3_nivel_zero.xlsx, DF4_validacao_recursiva.xlsx, DF5_simulacao_falha_06mar_0642_0742.xlsx, DF6_futuro_3h.xlsx) plus related plots (comparativo_12h.png updated, simulacao_falha_06mar_0642_0742.png updated, previsao_futura_2h.png added, previsao_futura_3h.png generated). Adds TODO.md describing the implementation plan and progress. Updates urt220.xlsx and urt221.xlsx (and adds backups urt220_old1.xlsx, urt221_old2.xlsx), and removes old UTR221_2025_2026_15MIN.xls copies.
</commit_message>
<xml_diff>
--- a/ML/DF5_simulacao_falha_06mar_0642_0742.xlsx
+++ b/ML/DF5_simulacao_falha_06mar_0642_0742.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,24 +45,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,39 +421,39 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Previsto_Recursivo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>BOMBA_1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>BOMBA_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NIVEL-UTR-220</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>46087.27916666667</v>
       </c>
       <c r="B2" t="n">
@@ -487,7 +473,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>46087.27986111111</v>
       </c>
       <c r="B3" t="n">
@@ -507,14 +493,14 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>46087.28055555555</v>
       </c>
       <c r="B4" t="n">
         <v>1.61</v>
       </c>
       <c r="C4" t="n">
-        <v>1.6103</v>
+        <v>1.6105</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -527,14 +513,14 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>46087.28125</v>
       </c>
       <c r="B5" t="n">
         <v>1.61</v>
       </c>
       <c r="C5" t="n">
-        <v>1.6101</v>
+        <v>1.6103</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -547,14 +533,14 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>46087.28194444445</v>
       </c>
       <c r="B6" t="n">
         <v>1.61</v>
       </c>
       <c r="C6" t="n">
-        <v>1.6121</v>
+        <v>1.6118</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -567,14 +553,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>46087.28263888889</v>
       </c>
       <c r="B7" t="n">
         <v>1.61</v>
       </c>
       <c r="C7" t="n">
-        <v>1.619</v>
+        <v>1.618</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -587,14 +573,14 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>46087.28333333333</v>
       </c>
       <c r="B8" t="n">
         <v>1.62</v>
       </c>
       <c r="C8" t="n">
-        <v>1.6201</v>
+        <v>1.6202</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -607,14 +593,14 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>46087.28402777778</v>
       </c>
       <c r="B9" t="n">
         <v>1.62</v>
       </c>
       <c r="C9" t="n">
-        <v>1.6211</v>
+        <v>1.6204</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
@@ -627,14 +613,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>46087.28472222222</v>
       </c>
       <c r="B10" t="n">
         <v>1.62</v>
       </c>
       <c r="C10" t="n">
-        <v>1.6213</v>
+        <v>1.621</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -647,14 +633,14 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>46087.28541666667</v>
       </c>
       <c r="B11" t="n">
         <v>1.62</v>
       </c>
       <c r="C11" t="n">
-        <v>1.6212</v>
+        <v>1.6213</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -667,14 +653,14 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>46087.28611111111</v>
       </c>
       <c r="B12" t="n">
         <v>1.62</v>
       </c>
       <c r="C12" t="n">
-        <v>1.6214</v>
+        <v>1.6216</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -687,14 +673,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>46087.28680555556</v>
       </c>
       <c r="B13" t="n">
         <v>1.62</v>
       </c>
       <c r="C13" t="n">
-        <v>1.6239</v>
+        <v>1.6219</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -707,14 +693,14 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>46087.2875</v>
       </c>
       <c r="B14" t="n">
         <v>1.62</v>
       </c>
       <c r="C14" t="n">
-        <v>1.6278</v>
+        <v>1.6251</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -727,14 +713,14 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>46087.28819444445</v>
       </c>
       <c r="B15" t="n">
         <v>1.62</v>
       </c>
       <c r="C15" t="n">
-        <v>1.63</v>
+        <v>1.6281</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -747,14 +733,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>46087.28888888889</v>
       </c>
       <c r="B16" t="n">
         <v>1.63</v>
       </c>
       <c r="C16" t="n">
-        <v>1.6321</v>
+        <v>1.6303</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -767,75 +753,75 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>46087.28958333333</v>
       </c>
       <c r="B17" t="n">
         <v>1.63</v>
       </c>
       <c r="C17" t="n">
+        <v>1.6305</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1.67</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>46087.29027777778</v>
+      </c>
+      <c r="B18" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1.6303</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.66</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>46087.29097222222</v>
+      </c>
+      <c r="B19" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1.6308</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.66</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>46087.29166666666</v>
+      </c>
+      <c r="B20" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="C20" t="n">
         <v>1.6309</v>
       </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>1.67</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>46087.29027777778</v>
-      </c>
-      <c r="B18" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="C18" t="n">
-        <v>1.6302</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="n">
-        <v>1.66</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>46087.29097222222</v>
-      </c>
-      <c r="B19" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="C19" t="n">
-        <v>1.6307</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>1.66</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>46087.29166666666</v>
-      </c>
-      <c r="B20" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="C20" t="n">
-        <v>1.6316</v>
-      </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
@@ -847,14 +833,14 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>46087.29236111111</v>
       </c>
       <c r="B21" t="n">
         <v>1.63</v>
       </c>
       <c r="C21" t="n">
-        <v>1.6364</v>
+        <v>1.6343</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -867,14 +853,14 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>46087.29305555556</v>
       </c>
       <c r="B22" t="n">
         <v>1.63</v>
       </c>
       <c r="C22" t="n">
-        <v>1.6407</v>
+        <v>1.6394</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -887,14 +873,14 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>46087.29375</v>
       </c>
       <c r="B23" t="n">
         <v>1.64</v>
       </c>
       <c r="C23" t="n">
-        <v>1.6404</v>
+        <v>1.64</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -907,14 +893,14 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>46087.29444444444</v>
       </c>
       <c r="B24" t="n">
         <v>1.64</v>
       </c>
       <c r="C24" t="n">
-        <v>1.6401</v>
+        <v>1.64</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -927,14 +913,14 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>46087.29513888889</v>
       </c>
       <c r="B25" t="n">
         <v>1.64</v>
       </c>
       <c r="C25" t="n">
-        <v>1.6404</v>
+        <v>1.6402</v>
       </c>
       <c r="D25" t="n">
         <v>1</v>
@@ -947,35 +933,35 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>46087.29583333333</v>
       </c>
       <c r="B26" t="n">
         <v>1.64</v>
       </c>
       <c r="C26" t="n">
+        <v>1.6403</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.63</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>46087.29652777778</v>
+      </c>
+      <c r="B27" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="C27" t="n">
         <v>1.6402</v>
       </c>
-      <c r="D26" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="n">
-        <v>1.63</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>46087.29652777778</v>
-      </c>
-      <c r="B27" t="n">
-        <v>1.64</v>
-      </c>
-      <c r="C27" t="n">
-        <v>1.6401</v>
-      </c>
       <c r="D27" t="n">
         <v>1</v>
       </c>
@@ -987,14 +973,14 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>46087.29722222222</v>
       </c>
       <c r="B28" t="n">
         <v>1.64</v>
       </c>
       <c r="C28" t="n">
-        <v>1.6445</v>
+        <v>1.6417</v>
       </c>
       <c r="D28" t="n">
         <v>1</v>
@@ -1007,14 +993,14 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>46087.29791666667</v>
       </c>
       <c r="B29" t="n">
         <v>1.64</v>
       </c>
       <c r="C29" t="n">
-        <v>1.6486</v>
+        <v>1.6471</v>
       </c>
       <c r="D29" t="n">
         <v>1</v>
@@ -1027,14 +1013,14 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>46087.29861111111</v>
       </c>
       <c r="B30" t="n">
         <v>1.65</v>
       </c>
       <c r="C30" t="n">
-        <v>1.6512</v>
+        <v>1.6502</v>
       </c>
       <c r="D30" t="n">
         <v>1</v>
@@ -1047,14 +1033,14 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>46087.29930555556</v>
       </c>
       <c r="B31" t="n">
         <v>1.65</v>
       </c>
       <c r="C31" t="n">
-        <v>1.6509</v>
+        <v>1.6511</v>
       </c>
       <c r="D31" t="n">
         <v>1</v>
@@ -1067,35 +1053,35 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>46087.3</v>
       </c>
       <c r="B32" t="n">
         <v>1.65</v>
       </c>
       <c r="C32" t="n">
+        <v>1.6501</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1.66</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>46087.30069444444</v>
+      </c>
+      <c r="B33" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C33" t="n">
         <v>1.6502</v>
       </c>
-      <c r="D32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" t="n">
-        <v>1.66</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>46087.30069444444</v>
-      </c>
-      <c r="B33" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1.6501</v>
-      </c>
       <c r="D33" t="n">
         <v>1</v>
       </c>
@@ -1107,14 +1093,14 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>46087.30138888889</v>
       </c>
       <c r="B34" t="n">
         <v>1.65</v>
       </c>
       <c r="C34" t="n">
-        <v>1.6511</v>
+        <v>1.651</v>
       </c>
       <c r="D34" t="n">
         <v>1</v>
@@ -1127,14 +1113,14 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>46087.30208333334</v>
       </c>
       <c r="B35" t="n">
         <v>1.65</v>
       </c>
       <c r="C35" t="n">
-        <v>1.6578</v>
+        <v>1.6561</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -1147,14 +1133,14 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>46087.30277777778</v>
       </c>
       <c r="B36" t="n">
         <v>1.65</v>
       </c>
       <c r="C36" t="n">
-        <v>1.66</v>
+        <v>1.657</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -1167,14 +1153,14 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>46087.30347222222</v>
       </c>
       <c r="B37" t="n">
         <v>1.66</v>
       </c>
       <c r="C37" t="n">
-        <v>1.6618</v>
+        <v>1.658</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -1187,14 +1173,14 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>46087.30416666667</v>
       </c>
       <c r="B38" t="n">
         <v>1.66</v>
       </c>
       <c r="C38" t="n">
-        <v>1.6601</v>
+        <v>1.66</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -1207,14 +1193,14 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>46087.30486111111</v>
       </c>
       <c r="B39" t="n">
         <v>1.66</v>
       </c>
       <c r="C39" t="n">
-        <v>1.6602</v>
+        <v>1.66</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -1227,14 +1213,14 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>46087.30555555555</v>
       </c>
       <c r="B40" t="n">
         <v>1.66</v>
       </c>
       <c r="C40" t="n">
-        <v>1.6608</v>
+        <v>1.662</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -1247,14 +1233,14 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>46087.30625</v>
       </c>
       <c r="B41" t="n">
         <v>1.66</v>
       </c>
       <c r="C41" t="n">
-        <v>1.6604</v>
+        <v>1.6607</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
@@ -1267,14 +1253,14 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>46087.30694444444</v>
       </c>
       <c r="B42" t="n">
         <v>1.66</v>
       </c>
       <c r="C42" t="n">
-        <v>1.6649</v>
+        <v>1.6609</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
@@ -1287,14 +1273,14 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>46087.30763888889</v>
       </c>
       <c r="B43" t="n">
         <v>1.66</v>
       </c>
       <c r="C43" t="n">
-        <v>1.6653</v>
+        <v>1.6659</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
@@ -1307,14 +1293,14 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>46087.30833333333</v>
       </c>
       <c r="B44" t="n">
         <v>1.67</v>
       </c>
       <c r="C44" t="n">
-        <v>1.6686</v>
+        <v>1.6658</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
@@ -1327,14 +1313,14 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>46087.30902777778</v>
       </c>
       <c r="B45" t="n">
         <v>1.67</v>
       </c>
       <c r="C45" t="n">
-        <v>1.6701</v>
+        <v>1.6681</v>
       </c>
       <c r="D45" t="n">
         <v>1</v>
@@ -1347,14 +1333,14 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>46087.30972222222</v>
       </c>
       <c r="B46" t="n">
         <v>1.67</v>
       </c>
       <c r="C46" t="n">
-        <v>1.6703</v>
+        <v>1.67</v>
       </c>
       <c r="D46" t="n">
         <v>1</v>
@@ -1367,14 +1353,14 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>46087.31041666667</v>
       </c>
       <c r="B47" t="n">
         <v>1.67</v>
       </c>
       <c r="C47" t="n">
-        <v>1.6712</v>
+        <v>1.67</v>
       </c>
       <c r="D47" t="n">
         <v>1</v>
@@ -1387,14 +1373,14 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>46087.31111111111</v>
       </c>
       <c r="B48" t="n">
         <v>1.67</v>
       </c>
       <c r="C48" t="n">
-        <v>1.6707</v>
+        <v>1.6702</v>
       </c>
       <c r="D48" t="n">
         <v>1</v>
@@ -1407,14 +1393,14 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>46087.31180555555</v>
       </c>
       <c r="B49" t="n">
         <v>1.67</v>
       </c>
       <c r="C49" t="n">
-        <v>1.6704</v>
+        <v>1.6716</v>
       </c>
       <c r="D49" t="n">
         <v>1</v>
@@ -1427,14 +1413,14 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>46087.3125</v>
       </c>
       <c r="B50" t="n">
         <v>1.67</v>
       </c>
       <c r="C50" t="n">
-        <v>1.673</v>
+        <v>1.6723</v>
       </c>
       <c r="D50" t="n">
         <v>1</v>
@@ -1447,14 +1433,14 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>46087.31319444445</v>
       </c>
       <c r="B51" t="n">
         <v>1.67</v>
       </c>
       <c r="C51" t="n">
-        <v>1.6777</v>
+        <v>1.6733</v>
       </c>
       <c r="D51" t="n">
         <v>1</v>
@@ -1467,14 +1453,14 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>46087.31388888889</v>
       </c>
       <c r="B52" t="n">
         <v>1.68</v>
       </c>
       <c r="C52" t="n">
-        <v>1.6794</v>
+        <v>1.676</v>
       </c>
       <c r="D52" t="n">
         <v>1</v>
@@ -1487,14 +1473,14 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>46087.31458333333</v>
       </c>
       <c r="B53" t="n">
         <v>1.68</v>
       </c>
       <c r="C53" t="n">
-        <v>1.6793</v>
+        <v>1.6795</v>
       </c>
       <c r="D53" t="n">
         <v>1</v>
@@ -1507,14 +1493,14 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>46087.31527777778</v>
       </c>
       <c r="B54" t="n">
         <v>1.68</v>
       </c>
       <c r="C54" t="n">
-        <v>1.6793</v>
+        <v>1.6798</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -1527,14 +1513,14 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>46087.31597222222</v>
       </c>
       <c r="B55" t="n">
         <v>1.68</v>
       </c>
       <c r="C55" t="n">
-        <v>1.676</v>
+        <v>1.6776</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
@@ -1547,14 +1533,14 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>46087.31666666667</v>
       </c>
       <c r="B56" t="n">
         <v>1.68</v>
       </c>
       <c r="C56" t="n">
-        <v>1.6767</v>
+        <v>1.6766</v>
       </c>
       <c r="D56" t="n">
         <v>0</v>
@@ -1567,14 +1553,14 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>46087.31736111111</v>
       </c>
       <c r="B57" t="n">
         <v>1.68</v>
       </c>
       <c r="C57" t="n">
-        <v>1.6815</v>
+        <v>1.68</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
@@ -1587,14 +1573,14 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>46087.31805555556</v>
       </c>
       <c r="B58" t="n">
         <v>1.68</v>
       </c>
       <c r="C58" t="n">
-        <v>1.6806</v>
+        <v>1.6794</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
@@ -1607,14 +1593,14 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>46087.31875</v>
       </c>
       <c r="B59" t="n">
         <v>1.68</v>
       </c>
       <c r="C59" t="n">
-        <v>1.6813</v>
+        <v>1.6802</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -1627,14 +1613,14 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>46087.31944444445</v>
       </c>
       <c r="B60" t="n">
         <v>1.68</v>
       </c>
       <c r="C60" t="n">
-        <v>1.6812</v>
+        <v>1.6838</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -1647,14 +1633,14 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>46087.32013888889</v>
       </c>
       <c r="B61" t="n">
         <v>1.68</v>
       </c>
       <c r="C61" t="n">
-        <v>1.6816</v>
+        <v>1.6827</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -1667,14 +1653,14 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>46087.32083333333</v>
       </c>
       <c r="B62" t="n">
         <v>1.69</v>
       </c>
       <c r="C62" t="n">
-        <v>1.6814</v>
+        <v>1.6802</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Add UTR221 ML simulation script and outputs
Introduce UTR221_ML_simulacao4.py: a full ML pipeline that loads urt220/urt221 data, performs feature engineering, trains RandomForest models, and runs recursive simulations (validation, failure simulation, future forecast and out-of-sample simulation). Exports multiple Excel dataframes (DF1_original, DF2_sem_zeros, DF3_nivel_zero, DF4_validacao_recursiva, DF5_simulacao_falha_06mar_0642_0742, DF6_futuro_3h, DF_simulacao.xlsx) and saves comparison/forecast/simulation plots (comparativo_12h.png, previsao_futura_3h.png, simulacao_falha_06mar_0642_0742.png, oos_simulacao_31mar.png). Adds TODO.md with implementation checklist and removes a transient LibreOffice lock file; updates several source xlsx and image binaries (including urt221.xlsx and related data files). Key behaviors: OOS window 31/03/2026 08:00-11:00, simulated communication failure 06/03/2026 06:42-07:42, and 3-hour recursive future forecast.
</commit_message>
<xml_diff>
--- a/ML/DF5_simulacao_falha_06mar_0642_0742.xlsx
+++ b/ML/DF5_simulacao_falha_06mar_0642_0742.xlsx
@@ -500,7 +500,7 @@
         <v>1.61</v>
       </c>
       <c r="C4" t="n">
-        <v>1.6104</v>
+        <v>1.6103</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -540,7 +540,7 @@
         <v>1.61</v>
       </c>
       <c r="C6" t="n">
-        <v>1.6124</v>
+        <v>1.6121</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -560,7 +560,7 @@
         <v>1.61</v>
       </c>
       <c r="C7" t="n">
-        <v>1.618</v>
+        <v>1.6182</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -620,7 +620,7 @@
         <v>1.62</v>
       </c>
       <c r="C10" t="n">
-        <v>1.6205</v>
+        <v>1.6204</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -640,7 +640,7 @@
         <v>1.62</v>
       </c>
       <c r="C11" t="n">
-        <v>1.6209</v>
+        <v>1.6207</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -660,7 +660,7 @@
         <v>1.62</v>
       </c>
       <c r="C12" t="n">
-        <v>1.622</v>
+        <v>1.6218</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -680,7 +680,7 @@
         <v>1.62</v>
       </c>
       <c r="C13" t="n">
-        <v>1.6222</v>
+        <v>1.6217</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -700,7 +700,7 @@
         <v>1.62</v>
       </c>
       <c r="C14" t="n">
-        <v>1.625</v>
+        <v>1.6251</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -720,7 +720,7 @@
         <v>1.62</v>
       </c>
       <c r="C15" t="n">
-        <v>1.6274</v>
+        <v>1.6276</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -740,7 +740,7 @@
         <v>1.63</v>
       </c>
       <c r="C16" t="n">
-        <v>1.6279</v>
+        <v>1.6307</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -760,7 +760,7 @@
         <v>1.63</v>
       </c>
       <c r="C17" t="n">
-        <v>1.631</v>
+        <v>1.6302</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -780,7 +780,7 @@
         <v>1.63</v>
       </c>
       <c r="C18" t="n">
-        <v>1.63</v>
+        <v>1.6306</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -800,7 +800,7 @@
         <v>1.63</v>
       </c>
       <c r="C19" t="n">
-        <v>1.6307</v>
+        <v>1.6305</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -820,7 +820,7 @@
         <v>1.63</v>
       </c>
       <c r="C20" t="n">
-        <v>1.6317</v>
+        <v>1.6318</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -840,7 +840,7 @@
         <v>1.63</v>
       </c>
       <c r="C21" t="n">
-        <v>1.6341</v>
+        <v>1.6346</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -860,7 +860,7 @@
         <v>1.63</v>
       </c>
       <c r="C22" t="n">
-        <v>1.6432</v>
+        <v>1.6397</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -880,7 +880,7 @@
         <v>1.64</v>
       </c>
       <c r="C23" t="n">
-        <v>1.6482</v>
+        <v>1.64</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -900,7 +900,7 @@
         <v>1.64</v>
       </c>
       <c r="C24" t="n">
-        <v>1.651</v>
+        <v>1.64</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -920,7 +920,7 @@
         <v>1.64</v>
       </c>
       <c r="C25" t="n">
-        <v>1.6504</v>
+        <v>1.6401</v>
       </c>
       <c r="D25" t="n">
         <v>1</v>
@@ -940,7 +940,7 @@
         <v>1.64</v>
       </c>
       <c r="C26" t="n">
-        <v>1.6512</v>
+        <v>1.6402</v>
       </c>
       <c r="D26" t="n">
         <v>1</v>
@@ -960,7 +960,7 @@
         <v>1.64</v>
       </c>
       <c r="C27" t="n">
-        <v>1.6511</v>
+        <v>1.6402</v>
       </c>
       <c r="D27" t="n">
         <v>1</v>
@@ -980,7 +980,7 @@
         <v>1.64</v>
       </c>
       <c r="C28" t="n">
-        <v>1.6529</v>
+        <v>1.6413</v>
       </c>
       <c r="D28" t="n">
         <v>1</v>
@@ -1000,7 +1000,7 @@
         <v>1.64</v>
       </c>
       <c r="C29" t="n">
-        <v>1.6579</v>
+        <v>1.6468</v>
       </c>
       <c r="D29" t="n">
         <v>1</v>
@@ -1020,7 +1020,7 @@
         <v>1.65</v>
       </c>
       <c r="C30" t="n">
-        <v>1.66</v>
+        <v>1.6501</v>
       </c>
       <c r="D30" t="n">
         <v>1</v>
@@ -1040,7 +1040,7 @@
         <v>1.65</v>
       </c>
       <c r="C31" t="n">
-        <v>1.6605</v>
+        <v>1.6511</v>
       </c>
       <c r="D31" t="n">
         <v>1</v>
@@ -1060,7 +1060,7 @@
         <v>1.65</v>
       </c>
       <c r="C32" t="n">
-        <v>1.6603</v>
+        <v>1.6503</v>
       </c>
       <c r="D32" t="n">
         <v>1</v>
@@ -1080,7 +1080,7 @@
         <v>1.65</v>
       </c>
       <c r="C33" t="n">
-        <v>1.6601</v>
+        <v>1.6507</v>
       </c>
       <c r="D33" t="n">
         <v>1</v>
@@ -1100,7 +1100,7 @@
         <v>1.65</v>
       </c>
       <c r="C34" t="n">
-        <v>1.661</v>
+        <v>1.6512</v>
       </c>
       <c r="D34" t="n">
         <v>1</v>
@@ -1120,7 +1120,7 @@
         <v>1.65</v>
       </c>
       <c r="C35" t="n">
-        <v>1.6609</v>
+        <v>1.6562</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -1140,7 +1140,7 @@
         <v>1.65</v>
       </c>
       <c r="C36" t="n">
-        <v>1.6608</v>
+        <v>1.6586</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -1160,7 +1160,7 @@
         <v>1.66</v>
       </c>
       <c r="C37" t="n">
-        <v>1.6602</v>
+        <v>1.6608</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -1200,7 +1200,7 @@
         <v>1.66</v>
       </c>
       <c r="C39" t="n">
-        <v>1.6603</v>
+        <v>1.66</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -1220,7 +1220,7 @@
         <v>1.66</v>
       </c>
       <c r="C40" t="n">
-        <v>1.6605</v>
+        <v>1.6619</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -1240,7 +1240,7 @@
         <v>1.66</v>
       </c>
       <c r="C41" t="n">
-        <v>1.664</v>
+        <v>1.6603</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
@@ -1260,7 +1260,7 @@
         <v>1.66</v>
       </c>
       <c r="C42" t="n">
-        <v>1.665</v>
+        <v>1.6639</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
@@ -1280,7 +1280,7 @@
         <v>1.66</v>
       </c>
       <c r="C43" t="n">
-        <v>1.6686</v>
+        <v>1.6649</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
@@ -1300,7 +1300,7 @@
         <v>1.67</v>
       </c>
       <c r="C44" t="n">
-        <v>1.6701</v>
+        <v>1.6666</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
@@ -1320,7 +1320,7 @@
         <v>1.67</v>
       </c>
       <c r="C45" t="n">
-        <v>1.6701</v>
+        <v>1.6685</v>
       </c>
       <c r="D45" t="n">
         <v>1</v>
@@ -1340,7 +1340,7 @@
         <v>1.67</v>
       </c>
       <c r="C46" t="n">
-        <v>1.6714</v>
+        <v>1.6703</v>
       </c>
       <c r="D46" t="n">
         <v>1</v>
@@ -1360,7 +1360,7 @@
         <v>1.67</v>
       </c>
       <c r="C47" t="n">
-        <v>1.6714</v>
+        <v>1.6701</v>
       </c>
       <c r="D47" t="n">
         <v>1</v>
@@ -1380,7 +1380,7 @@
         <v>1.67</v>
       </c>
       <c r="C48" t="n">
-        <v>1.6727</v>
+        <v>1.6702</v>
       </c>
       <c r="D48" t="n">
         <v>1</v>
@@ -1400,7 +1400,7 @@
         <v>1.67</v>
       </c>
       <c r="C49" t="n">
-        <v>1.6774</v>
+        <v>1.6715</v>
       </c>
       <c r="D49" t="n">
         <v>1</v>
@@ -1420,7 +1420,7 @@
         <v>1.67</v>
       </c>
       <c r="C50" t="n">
-        <v>1.6799</v>
+        <v>1.6747</v>
       </c>
       <c r="D50" t="n">
         <v>1</v>
@@ -1440,7 +1440,7 @@
         <v>1.67</v>
       </c>
       <c r="C51" t="n">
-        <v>1.6796</v>
+        <v>1.6764</v>
       </c>
       <c r="D51" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         <v>1.68</v>
       </c>
       <c r="C52" t="n">
-        <v>1.6798</v>
+        <v>1.6796</v>
       </c>
       <c r="D52" t="n">
         <v>1</v>
@@ -1480,7 +1480,7 @@
         <v>1.68</v>
       </c>
       <c r="C53" t="n">
-        <v>1.6775</v>
+        <v>1.6787</v>
       </c>
       <c r="D53" t="n">
         <v>1</v>
@@ -1500,7 +1500,7 @@
         <v>1.68</v>
       </c>
       <c r="C54" t="n">
-        <v>1.6767</v>
+        <v>1.6796</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -1520,7 +1520,7 @@
         <v>1.68</v>
       </c>
       <c r="C55" t="n">
-        <v>1.6795</v>
+        <v>1.6772</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
@@ -1540,7 +1540,7 @@
         <v>1.68</v>
       </c>
       <c r="C56" t="n">
-        <v>1.6795</v>
+        <v>1.6764</v>
       </c>
       <c r="D56" t="n">
         <v>0</v>
@@ -1580,7 +1580,7 @@
         <v>1.68</v>
       </c>
       <c r="C58" t="n">
-        <v>1.6824</v>
+        <v>1.6792</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
@@ -1600,7 +1600,7 @@
         <v>1.68</v>
       </c>
       <c r="C59" t="n">
-        <v>1.6807</v>
+        <v>1.6801</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -1620,7 +1620,7 @@
         <v>1.68</v>
       </c>
       <c r="C60" t="n">
-        <v>1.6811</v>
+        <v>1.6844</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -1640,7 +1640,7 @@
         <v>1.68</v>
       </c>
       <c r="C61" t="n">
-        <v>1.679</v>
+        <v>1.682</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -1660,7 +1660,7 @@
         <v>1.69</v>
       </c>
       <c r="C62" t="n">
-        <v>1.6775</v>
+        <v>1.68</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Add 7h future prediction and reorganize ML files
Introduce a new ML APP folder with data exports and a validation script (ML APP/UTR221_ML_validacao.py) that performs 1-min resampling, feature engineering and a recursive 7-hour (420 min) forecast, saving DF6_futuro_7h.xlsx and previsao_futura_7h.png. Add corresponding Excel/PNG assets and source data (urt220.xlsx, urt221.xlsx, DF* spreadsheets). Update ML/UTR221_ML_simulacao4.py to read S2 sensor columns and change the recursive prediction horizon to 3 hours. Remove several legacy/duplicated scripts and outdated forecast files from the ML root and update multiple DF Excel files and plots.
</commit_message>
<xml_diff>
--- a/ML/DF5_simulacao_falha_06mar_0642_0742.xlsx
+++ b/ML/DF5_simulacao_falha_06mar_0642_0742.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,13 +48,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,39 +435,39 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Previsto_Recursivo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>BOMBA_1</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>BOMBA_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>NIVEL-UTR-220</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>46087.27916666667</v>
       </c>
       <c r="B2" t="n">
@@ -466,261 +480,261 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>1.64</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>46087.27986111111</v>
       </c>
       <c r="B3" t="n">
         <v>1.61</v>
       </c>
       <c r="C3" t="n">
-        <v>1.61</v>
+        <v>1.6101</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>1.64</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>46087.28055555555</v>
       </c>
       <c r="B4" t="n">
         <v>1.61</v>
       </c>
       <c r="C4" t="n">
-        <v>1.6103</v>
+        <v>1.6107</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1.63</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>46087.28125</v>
       </c>
       <c r="B5" t="n">
         <v>1.61</v>
       </c>
       <c r="C5" t="n">
-        <v>1.6101</v>
+        <v>1.61</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>1.63</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>46087.28194444445</v>
       </c>
       <c r="B6" t="n">
         <v>1.61</v>
       </c>
       <c r="C6" t="n">
-        <v>1.6121</v>
+        <v>1.6122</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>1.63</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>46087.28263888889</v>
       </c>
       <c r="B7" t="n">
         <v>1.61</v>
       </c>
       <c r="C7" t="n">
-        <v>1.6182</v>
+        <v>1.619</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>1.63</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>46087.28333333333</v>
       </c>
       <c r="B8" t="n">
         <v>1.62</v>
       </c>
       <c r="C8" t="n">
-        <v>1.62</v>
+        <v>1.6206</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>1.63</v>
+        <v>3.27</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>46087.28402777778</v>
       </c>
       <c r="B9" t="n">
         <v>1.62</v>
       </c>
       <c r="C9" t="n">
-        <v>1.6204</v>
+        <v>1.6207</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>1.64</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>46087.28472222222</v>
       </c>
       <c r="B10" t="n">
         <v>1.62</v>
       </c>
       <c r="C10" t="n">
-        <v>1.6204</v>
+        <v>1.6213</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>1.65</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>46087.28541666667</v>
       </c>
       <c r="B11" t="n">
         <v>1.62</v>
       </c>
       <c r="C11" t="n">
-        <v>1.6207</v>
+        <v>1.6202</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>1.65</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>46087.28611111111</v>
       </c>
       <c r="B12" t="n">
         <v>1.62</v>
       </c>
       <c r="C12" t="n">
-        <v>1.6218</v>
+        <v>1.6201</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>1.66</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>46087.28680555556</v>
       </c>
       <c r="B13" t="n">
         <v>1.62</v>
       </c>
       <c r="C13" t="n">
-        <v>1.6217</v>
+        <v>1.6215</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>1.67</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>46087.2875</v>
       </c>
       <c r="B14" t="n">
         <v>1.62</v>
       </c>
       <c r="C14" t="n">
-        <v>1.6251</v>
+        <v>1.6233</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>46087.28819444445</v>
       </c>
       <c r="B15" t="n">
         <v>1.62</v>
       </c>
       <c r="C15" t="n">
-        <v>1.6276</v>
+        <v>1.6296</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -729,431 +743,431 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>1.67</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>46087.28888888889</v>
       </c>
       <c r="B16" t="n">
         <v>1.63</v>
       </c>
       <c r="C16" t="n">
-        <v>1.6307</v>
+        <v>1.63</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>1.67</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>46087.28958333333</v>
       </c>
       <c r="B17" t="n">
         <v>1.63</v>
       </c>
       <c r="C17" t="n">
-        <v>1.6302</v>
+        <v>1.6301</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>1.67</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>46087.29027777778</v>
       </c>
       <c r="B18" t="n">
         <v>1.63</v>
       </c>
       <c r="C18" t="n">
-        <v>1.6306</v>
+        <v>1.6303</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>1.66</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>46087.29097222222</v>
       </c>
       <c r="B19" t="n">
         <v>1.63</v>
       </c>
       <c r="C19" t="n">
-        <v>1.6305</v>
+        <v>1.63</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>1.66</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>46087.29166666666</v>
       </c>
       <c r="B20" t="n">
         <v>1.63</v>
       </c>
       <c r="C20" t="n">
-        <v>1.6318</v>
+        <v>1.6304</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>1.65</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>46087.29236111111</v>
       </c>
       <c r="B21" t="n">
         <v>1.63</v>
       </c>
       <c r="C21" t="n">
-        <v>1.6346</v>
+        <v>1.6317</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>1.65</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>46087.29305555556</v>
       </c>
       <c r="B22" t="n">
         <v>1.63</v>
       </c>
       <c r="C22" t="n">
-        <v>1.6397</v>
+        <v>1.6365</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>1.64</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>46087.29375</v>
       </c>
       <c r="B23" t="n">
         <v>1.64</v>
       </c>
       <c r="C23" t="n">
-        <v>1.64</v>
+        <v>1.6405</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>1.64</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>46087.29444444444</v>
       </c>
       <c r="B24" t="n">
         <v>1.64</v>
       </c>
       <c r="C24" t="n">
-        <v>1.64</v>
+        <v>1.6402</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>1.64</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>46087.29513888889</v>
       </c>
       <c r="B25" t="n">
         <v>1.64</v>
       </c>
       <c r="C25" t="n">
-        <v>1.6401</v>
+        <v>1.6406</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>1.63</v>
+        <v>3.27</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>46087.29583333333</v>
       </c>
       <c r="B26" t="n">
         <v>1.64</v>
       </c>
       <c r="C26" t="n">
-        <v>1.6402</v>
+        <v>1.6407</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>1.63</v>
+        <v>3.27</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>46087.29652777778</v>
       </c>
       <c r="B27" t="n">
         <v>1.64</v>
       </c>
       <c r="C27" t="n">
-        <v>1.6402</v>
+        <v>1.6407</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>1.63</v>
+        <v>3.27</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>46087.29722222222</v>
       </c>
       <c r="B28" t="n">
         <v>1.64</v>
       </c>
       <c r="C28" t="n">
-        <v>1.6413</v>
+        <v>1.6458</v>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28" t="n">
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>1.64</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>46087.29791666667</v>
       </c>
       <c r="B29" t="n">
         <v>1.64</v>
       </c>
       <c r="C29" t="n">
-        <v>1.6468</v>
+        <v>1.651</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>1.64</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>46087.29861111111</v>
       </c>
       <c r="B30" t="n">
         <v>1.65</v>
       </c>
       <c r="C30" t="n">
-        <v>1.6501</v>
+        <v>1.6526</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E30" t="n">
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>1.65</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>46087.29930555556</v>
       </c>
       <c r="B31" t="n">
         <v>1.65</v>
       </c>
       <c r="C31" t="n">
-        <v>1.6511</v>
+        <v>1.6583</v>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E31" t="n">
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>1.66</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>46087.3</v>
       </c>
       <c r="B32" t="n">
         <v>1.65</v>
       </c>
       <c r="C32" t="n">
-        <v>1.6503</v>
+        <v>1.66</v>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E32" t="n">
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>1.66</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>46087.30069444444</v>
       </c>
       <c r="B33" t="n">
         <v>1.65</v>
       </c>
       <c r="C33" t="n">
-        <v>1.6507</v>
+        <v>1.6608</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" t="n">
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>1.67</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>46087.30138888889</v>
       </c>
       <c r="B34" t="n">
         <v>1.65</v>
       </c>
       <c r="C34" t="n">
-        <v>1.6512</v>
+        <v>1.6604</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E34" t="n">
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>1.67</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>46087.30208333334</v>
       </c>
       <c r="B35" t="n">
         <v>1.65</v>
       </c>
       <c r="C35" t="n">
-        <v>1.6562</v>
+        <v>1.6609</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>1.67</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>46087.30277777778</v>
       </c>
       <c r="B36" t="n">
         <v>1.65</v>
       </c>
       <c r="C36" t="n">
-        <v>1.6586</v>
+        <v>1.6616</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>1.67</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>46087.30347222222</v>
       </c>
       <c r="B37" t="n">
@@ -1166,341 +1180,341 @@
         <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>1.66</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>46087.30416666667</v>
       </c>
       <c r="B38" t="n">
         <v>1.66</v>
       </c>
       <c r="C38" t="n">
-        <v>1.66</v>
+        <v>1.6604</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>1.66</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>46087.30486111111</v>
       </c>
       <c r="B39" t="n">
         <v>1.66</v>
       </c>
       <c r="C39" t="n">
-        <v>1.66</v>
+        <v>1.6605</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>1.66</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>46087.30555555555</v>
       </c>
       <c r="B40" t="n">
         <v>1.66</v>
       </c>
       <c r="C40" t="n">
-        <v>1.6619</v>
+        <v>1.6604</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>1.65</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>46087.30625</v>
       </c>
       <c r="B41" t="n">
         <v>1.66</v>
       </c>
       <c r="C41" t="n">
-        <v>1.6603</v>
+        <v>1.6615</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
       </c>
       <c r="E41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>1.65</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>46087.30694444444</v>
       </c>
       <c r="B42" t="n">
         <v>1.66</v>
       </c>
       <c r="C42" t="n">
-        <v>1.6639</v>
+        <v>1.6631</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>1.64</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>46087.30763888889</v>
       </c>
       <c r="B43" t="n">
         <v>1.66</v>
       </c>
       <c r="C43" t="n">
-        <v>1.6649</v>
+        <v>1.6682</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>1.64</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>46087.30833333333</v>
       </c>
       <c r="B44" t="n">
         <v>1.67</v>
       </c>
       <c r="C44" t="n">
-        <v>1.6666</v>
+        <v>1.67</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>1.64</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>46087.30902777778</v>
       </c>
       <c r="B45" t="n">
         <v>1.67</v>
       </c>
       <c r="C45" t="n">
-        <v>1.6685</v>
+        <v>1.6703</v>
       </c>
       <c r="D45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>1.63</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>46087.30972222222</v>
       </c>
       <c r="B46" t="n">
         <v>1.67</v>
       </c>
       <c r="C46" t="n">
-        <v>1.6703</v>
+        <v>1.6702</v>
       </c>
       <c r="D46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>1.63</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>46087.31041666667</v>
       </c>
       <c r="B47" t="n">
         <v>1.67</v>
       </c>
       <c r="C47" t="n">
-        <v>1.6701</v>
+        <v>1.6705</v>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>1.63</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>46087.31111111111</v>
       </c>
       <c r="B48" t="n">
         <v>1.67</v>
       </c>
       <c r="C48" t="n">
-        <v>1.6702</v>
+        <v>1.6715</v>
       </c>
       <c r="D48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E48" t="n">
         <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>1.63</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>46087.31180555555</v>
       </c>
       <c r="B49" t="n">
         <v>1.67</v>
       </c>
       <c r="C49" t="n">
-        <v>1.6715</v>
+        <v>1.6735</v>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E49" t="n">
         <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>1.64</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>46087.3125</v>
       </c>
       <c r="B50" t="n">
         <v>1.67</v>
       </c>
       <c r="C50" t="n">
-        <v>1.6747</v>
+        <v>1.6783</v>
       </c>
       <c r="D50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E50" t="n">
         <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>1.65</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>46087.31319444445</v>
       </c>
       <c r="B51" t="n">
         <v>1.67</v>
       </c>
       <c r="C51" t="n">
-        <v>1.6764</v>
+        <v>1.6801</v>
       </c>
       <c r="D51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E51" t="n">
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>1.65</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>46087.31388888889</v>
       </c>
       <c r="B52" t="n">
         <v>1.68</v>
       </c>
       <c r="C52" t="n">
-        <v>1.6796</v>
+        <v>1.6802</v>
       </c>
       <c r="D52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E52" t="n">
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>1.66</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>46087.31458333333</v>
       </c>
       <c r="B53" t="n">
         <v>1.68</v>
       </c>
       <c r="C53" t="n">
-        <v>1.6787</v>
+        <v>1.6804</v>
       </c>
       <c r="D53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E53" t="n">
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>1.67</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>46087.31527777778</v>
       </c>
       <c r="B54" t="n">
         <v>1.68</v>
       </c>
       <c r="C54" t="n">
-        <v>1.6796</v>
+        <v>1.6806</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -1509,167 +1523,167 @@
         <v>1</v>
       </c>
       <c r="F54" t="n">
-        <v>1.67</v>
+        <v>3.16</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>46087.31597222222</v>
       </c>
       <c r="B55" t="n">
         <v>1.68</v>
       </c>
       <c r="C55" t="n">
-        <v>1.6772</v>
+        <v>1.6801</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
       </c>
       <c r="E55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F55" t="n">
-        <v>1.67</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>46087.31666666667</v>
       </c>
       <c r="B56" t="n">
         <v>1.68</v>
       </c>
       <c r="C56" t="n">
-        <v>1.6764</v>
+        <v>1.6813</v>
       </c>
       <c r="D56" t="n">
         <v>0</v>
       </c>
       <c r="E56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>1.66</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>46087.31736111111</v>
       </c>
       <c r="B57" t="n">
         <v>1.68</v>
       </c>
       <c r="C57" t="n">
-        <v>1.6803</v>
+        <v>1.6808</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
       </c>
       <c r="E57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F57" t="n">
-        <v>1.66</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>46087.31805555556</v>
       </c>
       <c r="B58" t="n">
         <v>1.68</v>
       </c>
       <c r="C58" t="n">
-        <v>1.6792</v>
+        <v>1.6801</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
       </c>
       <c r="E58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>1.66</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>46087.31875</v>
       </c>
       <c r="B59" t="n">
         <v>1.68</v>
       </c>
       <c r="C59" t="n">
-        <v>1.6801</v>
+        <v>1.6825</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>1.65</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>46087.31944444445</v>
       </c>
       <c r="B60" t="n">
         <v>1.68</v>
       </c>
       <c r="C60" t="n">
-        <v>1.6844</v>
+        <v>1.6825</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
       </c>
       <c r="E60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F60" t="n">
-        <v>1.65</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>46087.32013888889</v>
       </c>
       <c r="B61" t="n">
         <v>1.68</v>
       </c>
       <c r="C61" t="n">
-        <v>1.682</v>
+        <v>1.6855</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
       </c>
       <c r="E61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F61" t="n">
-        <v>1.64</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>46087.32083333333</v>
       </c>
       <c r="B62" t="n">
         <v>1.69</v>
       </c>
       <c r="C62" t="n">
-        <v>1.68</v>
+        <v>1.6852</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
       </c>
       <c r="E62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>1.64</v>
+        <v>3.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>